<commit_message>
Update paytable values and add new symbol for RB in gameconfig004
</commit_message>
<xml_diff>
--- a/assets/gamecfg004/paytable.xlsx
+++ b/assets/gamecfg004/paytable.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="27">
   <si>
     <t>Code</t>
   </si>
@@ -86,6 +86,12 @@
   </si>
   <si>
     <t>L4</t>
+  </si>
+  <si>
+    <t>9</t>
+  </si>
+  <si>
+    <t>RB</t>
   </si>
 </sst>
 </file>
@@ -1254,7 +1260,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr defaultColWidth="8" defaultRowHeight="12.75" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="7" width="8" style="1" customWidth="1"/>
@@ -1298,13 +1304,13 @@
         <v>0</v>
       </c>
       <c r="E2" s="3">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="F2" s="4">
-        <v>400</v>
+        <v>300</v>
       </c>
       <c r="G2" s="3">
-        <v>2000</v>
+        <v>1600</v>
       </c>
     </row>
     <row r="3" ht="15.35" customHeight="1">
@@ -1489,6 +1495,29 @@
       </c>
       <c r="G10" s="3">
         <v>160</v>
+      </c>
+    </row>
+    <row r="11" ht="15.35" customHeight="1">
+      <c r="A11" t="s" s="2">
+        <v>25</v>
+      </c>
+      <c r="B11" t="s" s="2">
+        <v>26</v>
+      </c>
+      <c r="C11" s="3">
+        <v>0</v>
+      </c>
+      <c r="D11" s="4">
+        <v>0</v>
+      </c>
+      <c r="E11" s="3">
+        <v>80</v>
+      </c>
+      <c r="F11" s="4">
+        <v>400</v>
+      </c>
+      <c r="G11" s="3">
+        <v>2000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(gameconfig): add new symbols and payouts for RB2 to RB5
</commit_message>
<xml_diff>
--- a/assets/gamecfg004/paytable.xlsx
+++ b/assets/gamecfg004/paytable.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="35">
   <si>
     <t>Code</t>
   </si>
@@ -92,6 +92,30 @@
   </si>
   <si>
     <t>RB</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>RB2</t>
+  </si>
+  <si>
+    <t>11</t>
+  </si>
+  <si>
+    <t>RB3</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>RB4</t>
+  </si>
+  <si>
+    <t>13</t>
+  </si>
+  <si>
+    <t>RB5</t>
   </si>
 </sst>
 </file>
@@ -1260,7 +1284,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr defaultColWidth="8" defaultRowHeight="12.75" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="7" width="8" style="1" customWidth="1"/>
@@ -1517,6 +1541,98 @@
         <v>400</v>
       </c>
       <c r="G11" s="3">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="12" ht="15.35" customHeight="1">
+      <c r="A12" t="s" s="2">
+        <v>27</v>
+      </c>
+      <c r="B12" t="s" s="2">
+        <v>28</v>
+      </c>
+      <c r="C12" s="3">
+        <v>0</v>
+      </c>
+      <c r="D12" s="4">
+        <v>0</v>
+      </c>
+      <c r="E12" s="3">
+        <v>80</v>
+      </c>
+      <c r="F12" s="4">
+        <v>400</v>
+      </c>
+      <c r="G12" s="3">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="13" ht="15.35" customHeight="1">
+      <c r="A13" t="s" s="2">
+        <v>29</v>
+      </c>
+      <c r="B13" t="s" s="2">
+        <v>30</v>
+      </c>
+      <c r="C13" s="3">
+        <v>0</v>
+      </c>
+      <c r="D13" s="4">
+        <v>0</v>
+      </c>
+      <c r="E13" s="3">
+        <v>80</v>
+      </c>
+      <c r="F13" s="4">
+        <v>400</v>
+      </c>
+      <c r="G13" s="3">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="14" ht="15.35" customHeight="1">
+      <c r="A14" t="s" s="2">
+        <v>31</v>
+      </c>
+      <c r="B14" t="s" s="2">
+        <v>32</v>
+      </c>
+      <c r="C14" s="3">
+        <v>0</v>
+      </c>
+      <c r="D14" s="4">
+        <v>0</v>
+      </c>
+      <c r="E14" s="3">
+        <v>80</v>
+      </c>
+      <c r="F14" s="4">
+        <v>400</v>
+      </c>
+      <c r="G14" s="3">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="15" ht="15.35" customHeight="1">
+      <c r="A15" t="s" s="2">
+        <v>33</v>
+      </c>
+      <c r="B15" t="s" s="2">
+        <v>34</v>
+      </c>
+      <c r="C15" s="3">
+        <v>0</v>
+      </c>
+      <c r="D15" s="4">
+        <v>0</v>
+      </c>
+      <c r="E15" s="3">
+        <v>80</v>
+      </c>
+      <c r="F15" s="4">
+        <v>400</v>
+      </c>
+      <c r="G15" s="3">
         <v>2000</v>
       </c>
     </row>

</xml_diff>